<commit_message>
chore: update pre-1997 workbook artifact
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/early_data/out/footbag_results_pre1997_v1.xlsx
+++ b/early_data/out/footbag_results_pre1997_v1.xlsx
@@ -26208,7 +26208,7 @@
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>Women's Dbls Net</t>
+          <t>Mixed Doubles Net</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
@@ -26278,7 +26278,7 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>Open Sgls Consecutiv</t>
+          <t>Open Dbls Consecutiv</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
@@ -26313,7 +26313,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Ultra Doubles Net</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -26348,7 +26348,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Doubles Net</t>
+          <t>Mixed Doubles Net</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -26418,7 +26418,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Doubles Net</t>
+          <t>Open Dbls Net</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
@@ -26519,7 +26519,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Women's Dbls Net</t>
+          <t>Women's Sgls Net</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -26589,7 +26589,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Women's Dbls Net</t>
+          <t>Mixed Doubles Net</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -26624,7 +26624,7 @@
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>Golf</t>
+          <t>Open Dbls Consecutiv</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
@@ -26694,7 +26694,7 @@
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>Women's Doubles Cons</t>
+          <t>Mixed Doubles Net</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
@@ -26764,7 +26764,7 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>Doubles Net</t>
+          <t>Singles Net</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
@@ -26799,7 +26799,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Open Sgls Net</t>
+          <t>Open Dbls Consecutiv</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -26834,7 +26834,7 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Mixed Doubles Net</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
@@ -26869,7 +26869,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Open Dbls Consecutiv</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -27009,7 +27009,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Doubles Net</t>
+          <t>Open Dbls Net</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -27145,7 +27145,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Doubles Net</t>
+          <t>Open Dbls Net</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -27347,7 +27347,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doubles Consecutive </t>
+          <t>Singles</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -27417,7 +27417,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Women's Dbls Net</t>
+          <t>Women's Freestyle</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -27452,7 +27452,7 @@
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Mixed Doubles Net</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr">
@@ -27487,7 +27487,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Mixed Doubles Net</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -27522,7 +27522,7 @@
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doubles Consecutive </t>
+          <t>Advanced Doubles Net</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
@@ -27592,7 +27592,7 @@
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>Women's Dbls Net</t>
+          <t>Women's Sgls Net</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
@@ -27697,7 +27697,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Doubles Net</t>
+          <t>Open Singles Net</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -27732,7 +27732,7 @@
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Open Dbls Consecutiv</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
@@ -27767,7 +27767,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Women's Doubles Net</t>
+          <t>Mixed Dbls Net</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -27802,7 +27802,7 @@
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>Team Consecutive Kic</t>
+          <t>Women's Singles Cons</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
@@ -27872,7 +27872,7 @@
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>Women's Singles Net</t>
+          <t>Women's Sgls Net</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
@@ -27942,7 +27942,7 @@
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>Open Doubles Net</t>
+          <t>Open Singles</t>
         </is>
       </c>
       <c r="G52" s="8" t="inlineStr">
@@ -28012,7 +28012,7 @@
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Doubles Net</t>
         </is>
       </c>
       <c r="G54" s="8" t="inlineStr">
@@ -28152,7 +28152,7 @@
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>Women's Freestyle</t>
+          <t>Women's Team Freesty</t>
         </is>
       </c>
       <c r="G58" s="8" t="inlineStr">
@@ -28222,7 +28222,7 @@
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>Women's Dbls Net</t>
+          <t>Women's Golf</t>
         </is>
       </c>
       <c r="G60" s="8" t="inlineStr">
@@ -28257,7 +28257,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Women's Dbls Net</t>
+          <t>Mixed Doubles Net</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -28292,7 +28292,7 @@
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Mixed Doubles Net</t>
         </is>
       </c>
       <c r="G62" s="8" t="inlineStr">
@@ -28327,7 +28327,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Women's Doubles Cons</t>
+          <t>Women's Singles Cons</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -28432,7 +28432,7 @@
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t>Doubles Net</t>
+          <t>Intermediate Singles</t>
         </is>
       </c>
       <c r="G66" s="8" t="inlineStr">
@@ -28467,7 +28467,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Golf</t>
+          <t>Ultra Doubles Net</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -28502,7 +28502,7 @@
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>Open Doubles</t>
+          <t>Open Singles</t>
         </is>
       </c>
       <c r="G68" s="8" t="inlineStr">
@@ -28572,7 +28572,7 @@
       </c>
       <c r="F70" s="8" t="inlineStr">
         <is>
-          <t>Doubles Net</t>
+          <t>Open Dbls Net</t>
         </is>
       </c>
       <c r="G70" s="8" t="inlineStr">
@@ -28642,7 +28642,7 @@
       </c>
       <c r="F72" s="8" t="inlineStr">
         <is>
-          <t>Women's Doubles Cons</t>
+          <t>Women's Sgls Freesty</t>
         </is>
       </c>
       <c r="G72" s="8" t="inlineStr">
@@ -28677,7 +28677,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doubles Consecutive </t>
+          <t>Open Sgls Consecutiv</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -28883,7 +28883,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Open Freestyle</t>
+          <t>Open Sgls Consecutiv</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -28918,7 +28918,7 @@
       </c>
       <c r="F80" s="8" t="inlineStr">
         <is>
-          <t>Women's Dbls Net</t>
+          <t>Mixed Doubles Net</t>
         </is>
       </c>
       <c r="G80" s="8" t="inlineStr">
@@ -28953,7 +28953,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Open Team Freestyle</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -28988,7 +28988,7 @@
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
-          <t>Women's Doubles One-</t>
+          <t>Women's Team Freesty</t>
         </is>
       </c>
       <c r="G82" s="8" t="inlineStr">
@@ -29023,7 +29023,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Ultra Doubles Net</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -29058,7 +29058,7 @@
       </c>
       <c r="F84" s="8" t="inlineStr">
         <is>
-          <t>Women's Dbls Net</t>
+          <t>Mixed Doubles Net</t>
         </is>
       </c>
       <c r="G84" s="8" t="inlineStr">
@@ -29198,7 +29198,7 @@
       </c>
       <c r="F88" s="8" t="inlineStr">
         <is>
-          <t>Open Sgls Net</t>
+          <t>Open Singles Net</t>
         </is>
       </c>
       <c r="G88" s="8" t="inlineStr">
@@ -29268,7 +29268,7 @@
       </c>
       <c r="F90" s="8" t="inlineStr">
         <is>
-          <t>Women's Team Freesty</t>
+          <t>Women's Dbls Net</t>
         </is>
       </c>
       <c r="G90" s="8" t="inlineStr">
@@ -29478,7 +29478,7 @@
       </c>
       <c r="F96" s="8" t="inlineStr">
         <is>
-          <t>Open Golf</t>
+          <t>Intermediate Doubles</t>
         </is>
       </c>
       <c r="G96" s="8" t="inlineStr">
@@ -29513,7 +29513,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Open Sgls Freestyle</t>
+          <t>Open Team Freestyle</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -29548,7 +29548,7 @@
       </c>
       <c r="F98" s="8" t="inlineStr">
         <is>
-          <t>Women's Doubles Cons</t>
+          <t>Mixed Doubles Net</t>
         </is>
       </c>
       <c r="G98" s="8" t="inlineStr">
@@ -29583,7 +29583,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Women's Dbls Net</t>
+          <t>Mixed Doubles Net</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -29618,7 +29618,7 @@
       </c>
       <c r="F100" s="8" t="inlineStr">
         <is>
-          <t>Women's Doubles Cons</t>
+          <t>Women's Freestyle</t>
         </is>
       </c>
       <c r="G100" s="8" t="inlineStr">
@@ -29653,7 +29653,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Doubles Net</t>
+          <t>Singles Net</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -29688,7 +29688,7 @@
       </c>
       <c r="F102" s="8" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Open Team Freestyle</t>
         </is>
       </c>
       <c r="G102" s="8" t="inlineStr">

</xml_diff>